<commit_message>
New P fertiliser file
</commit_message>
<xml_diff>
--- a/data-preprocessing/rpc-footprints/1 - Crops/P fertiliser.xlsx
+++ b/data-preprocessing/rpc-footprints/1 - Crops/P fertiliser.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" updateLinks="never" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75532E07-6E21-F347-B3F2-CD5C65A60D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFA6C3EB-7AA7-4ABB-8783-A468D5FE703C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INFO" sheetId="117" r:id="rId1"/>
@@ -30,6 +30,7 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1831" uniqueCount="745">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1842" uniqueCount="747">
   <si>
     <t>Crops</t>
   </si>
@@ -2364,6 +2365,12 @@
   <si>
     <t>Default-01229</t>
   </si>
+  <si>
+    <t>Yara (2018). Gödslingsråd. https://www.yara.se/contentassets/b2d039536ac14ce382a98e12dd92282e/yar0050_godslingsradet_2018_okt.pdf</t>
+  </si>
+  <si>
+    <t>Yara (2018)</t>
+  </si>
 </sst>
 </file>
 
@@ -2373,7 +2380,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2518,8 +2525,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2541,12 +2555,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2576,7 +2584,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2710,9 +2718,10 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="1" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="12">
     <cellStyle name="Hyperlink" xfId="10" xr:uid="{5049D40D-41C5-449C-992D-6D555AE79C87}"/>
@@ -3013,30 +3022,30 @@
     <tabColor theme="1"/>
   </sheetPr>
   <dimension ref="A2:G19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="27.33203125" customWidth="1"/>
+    <col min="2" max="2" width="27.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" ht="21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="21" x14ac:dyDescent="0.5">
       <c r="A2" s="3" t="s">
         <v>651</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>650</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A6" s="27" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A7" s="27"/>
     </row>
-    <row r="8" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="28" t="s">
         <v>1</v>
       </c>
@@ -3050,7 +3059,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -3067,7 +3076,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -3084,7 +3093,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -3101,7 +3110,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -3118,7 +3127,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>76</v>
       </c>
@@ -3135,7 +3144,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>58</v>
       </c>
@@ -3149,7 +3158,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
         <v>638</v>
       </c>
@@ -3163,7 +3172,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>637</v>
       </c>
@@ -3178,7 +3187,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>639</v>
       </c>
@@ -3202,22 +3211,22 @@
     <tabColor theme="6" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A2:GT115"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.33203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="175" width="5.6640625" customWidth="1"/>
-    <col min="176" max="176" width="5.6640625" style="1" customWidth="1"/>
-    <col min="177" max="202" width="5.6640625" customWidth="1"/>
+    <col min="2" max="2" width="32.90625" customWidth="1"/>
+    <col min="3" max="3" width="15.36328125" customWidth="1"/>
+    <col min="4" max="4" width="15.81640625" customWidth="1"/>
+    <col min="5" max="175" width="5.6328125" customWidth="1"/>
+    <col min="176" max="176" width="5.6328125" style="1" customWidth="1"/>
+    <col min="177" max="202" width="5.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:202" ht="19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:202" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A2" s="20" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="4" spans="1:202" ht="78.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:202" ht="78.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
@@ -3818,7 +3827,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="5" spans="1:202" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:202" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="31" t="s">
         <v>1</v>
       </c>
@@ -4426,7 +4435,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="6" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -4457,7 +4466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -4472,7 +4481,7 @@
       </c>
       <c r="FT7" s="53"/>
     </row>
-    <row r="8" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -4492,7 +4501,7 @@
         <v>6.0001458928005071</v>
       </c>
     </row>
-    <row r="9" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -4507,7 +4516,7 @@
       </c>
       <c r="FT9" s="53"/>
     </row>
-    <row r="10" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -4525,7 +4534,7 @@
       </c>
       <c r="FT10" s="53"/>
     </row>
-    <row r="11" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -4545,7 +4554,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -4564,7 +4573,7 @@
       </c>
       <c r="FT12" s="53"/>
     </row>
-    <row r="13" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -4594,7 +4603,7 @@
       </c>
       <c r="FT13" s="53"/>
     </row>
-    <row r="14" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -4614,7 +4623,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -4634,7 +4643,7 @@
         <v>6.9999999999999991</v>
       </c>
     </row>
-    <row r="16" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -4654,7 +4663,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
@@ -4674,7 +4683,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
@@ -4692,7 +4701,7 @@
       </c>
       <c r="FT18" s="54"/>
     </row>
-    <row r="19" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
@@ -4707,7 +4716,7 @@
       </c>
       <c r="FT19" s="53"/>
     </row>
-    <row r="20" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
@@ -4727,7 +4736,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>19</v>
       </c>
@@ -4743,9 +4752,12 @@
       <c r="BC21">
         <v>32</v>
       </c>
-      <c r="FT21" s="54"/>
-    </row>
-    <row r="22" spans="1:176" x14ac:dyDescent="0.2">
+      <c r="FT21" s="59">
+        <f>AVERAGE(20,40)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -4761,11 +4773,12 @@
       <c r="BC22">
         <v>40</v>
       </c>
-      <c r="FT22" s="54">
-        <v>22.944752181740999</v>
-      </c>
-    </row>
-    <row r="23" spans="1:176" x14ac:dyDescent="0.2">
+      <c r="FT22" s="59">
+        <f>AVERAGE(20,40)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>21</v>
       </c>
@@ -4779,7 +4792,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="24" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>22</v>
       </c>
@@ -4795,11 +4808,12 @@
       <c r="BC24">
         <v>40</v>
       </c>
-      <c r="FT24" s="53">
-        <v>16.000028640472568</v>
-      </c>
-    </row>
-    <row r="25" spans="1:176" x14ac:dyDescent="0.2">
+      <c r="FT24" s="60">
+        <f>AVERAGE(30,50)</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
@@ -4816,7 +4830,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
@@ -4832,11 +4846,12 @@
       <c r="BC26">
         <v>35</v>
       </c>
-      <c r="FT26" s="54">
-        <v>29.745999999999999</v>
-      </c>
-    </row>
-    <row r="27" spans="1:176" x14ac:dyDescent="0.2">
+      <c r="FT26" s="59">
+        <f>AVERAGE(30,60)</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="27" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
@@ -4854,7 +4869,7 @@
         <v>60.578214285714289</v>
       </c>
     </row>
-    <row r="28" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
@@ -4871,11 +4886,12 @@
         <v>40</v>
       </c>
       <c r="FP28" s="25"/>
-      <c r="FT28" s="54">
-        <v>21.384</v>
-      </c>
-    </row>
-    <row r="29" spans="1:176" x14ac:dyDescent="0.2">
+      <c r="FT28" s="59">
+        <f>AVERAGE(20,40)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="29" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
@@ -4888,11 +4904,12 @@
       <c r="D29" t="s">
         <v>401</v>
       </c>
-      <c r="FT29" s="53">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="30" spans="1:176" x14ac:dyDescent="0.2">
+      <c r="FT29" s="59">
+        <f>AVERAGE(20,40)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
@@ -4908,7 +4925,7 @@
       <c r="M30" s="25"/>
       <c r="FT30" s="54"/>
     </row>
-    <row r="31" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>29</v>
       </c>
@@ -4923,7 +4940,7 @@
       </c>
       <c r="FT31" s="54"/>
     </row>
-    <row r="32" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>30</v>
       </c>
@@ -4938,7 +4955,7 @@
       </c>
       <c r="FT32" s="53"/>
     </row>
-    <row r="33" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>31</v>
       </c>
@@ -4956,7 +4973,7 @@
       </c>
       <c r="FT33" s="53"/>
     </row>
-    <row r="34" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
@@ -4981,7 +4998,7 @@
       </c>
       <c r="FT34" s="53"/>
     </row>
-    <row r="35" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>33</v>
       </c>
@@ -5009,7 +5026,7 @@
       </c>
       <c r="FT35" s="53"/>
     </row>
-    <row r="36" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>34</v>
       </c>
@@ -5037,7 +5054,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="37" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>35</v>
       </c>
@@ -5057,7 +5074,7 @@
         <v>703.72159999999997</v>
       </c>
     </row>
-    <row r="38" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>36</v>
       </c>
@@ -5077,7 +5094,7 @@
         <v>36.184615384615398</v>
       </c>
     </row>
-    <row r="39" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>37</v>
       </c>
@@ -5097,7 +5114,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="40" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>38</v>
       </c>
@@ -5112,7 +5129,7 @@
       </c>
       <c r="FT40" s="54"/>
     </row>
-    <row r="41" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>39</v>
       </c>
@@ -5130,7 +5147,7 @@
       </c>
       <c r="FT41" s="54"/>
     </row>
-    <row r="42" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>40</v>
       </c>
@@ -5145,7 +5162,7 @@
       </c>
       <c r="FT42" s="54"/>
     </row>
-    <row r="43" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>41</v>
       </c>
@@ -5160,7 +5177,7 @@
       </c>
       <c r="FT43" s="54"/>
     </row>
-    <row r="44" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>42</v>
       </c>
@@ -5175,7 +5192,7 @@
       </c>
       <c r="FT44" s="54"/>
     </row>
-    <row r="45" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>43</v>
       </c>
@@ -5192,7 +5209,7 @@
         <v>2.6518741381471731</v>
       </c>
     </row>
-    <row r="46" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>44</v>
       </c>
@@ -5207,7 +5224,7 @@
       </c>
       <c r="FT46" s="54"/>
     </row>
-    <row r="47" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>45</v>
       </c>
@@ -5224,7 +5241,7 @@
         <v>3.4794938917975569</v>
       </c>
     </row>
-    <row r="48" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>46</v>
       </c>
@@ -5249,7 +5266,7 @@
       </c>
       <c r="FT48" s="54"/>
     </row>
-    <row r="49" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>47</v>
       </c>
@@ -5264,7 +5281,7 @@
       </c>
       <c r="FT49" s="54"/>
     </row>
-    <row r="50" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>48</v>
       </c>
@@ -5283,7 +5300,7 @@
       </c>
       <c r="FT50" s="54"/>
     </row>
-    <row r="51" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>49</v>
       </c>
@@ -5299,11 +5316,12 @@
       <c r="BC51">
         <v>35</v>
       </c>
-      <c r="FT51" s="54">
-        <v>43.999849495467764</v>
-      </c>
-    </row>
-    <row r="52" spans="1:176" x14ac:dyDescent="0.2">
+      <c r="FT51" s="59">
+        <f>AVERAGE(40,80)</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="52" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>50</v>
       </c>
@@ -5321,7 +5339,7 @@
       </c>
       <c r="FT52" s="54"/>
     </row>
-    <row r="53" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>51</v>
       </c>
@@ -5338,7 +5356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>52</v>
       </c>
@@ -5354,11 +5372,12 @@
       <c r="BC54">
         <v>30</v>
       </c>
-      <c r="FT54" s="54">
-        <v>20.999786788501808</v>
-      </c>
-    </row>
-    <row r="55" spans="1:176" x14ac:dyDescent="0.2">
+      <c r="FT54" s="59">
+        <f>AVERAGE(20,60)</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="55" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>53</v>
       </c>
@@ -5375,7 +5394,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="56" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>54</v>
       </c>
@@ -5393,7 +5412,7 @@
       </c>
       <c r="FT56" s="54"/>
     </row>
-    <row r="57" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>55</v>
       </c>
@@ -5413,7 +5432,7 @@
         <v>36.999160363086233</v>
       </c>
     </row>
-    <row r="58" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>56</v>
       </c>
@@ -5432,7 +5451,7 @@
       </c>
       <c r="FT58" s="54"/>
     </row>
-    <row r="59" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>57</v>
       </c>
@@ -5450,7 +5469,7 @@
       </c>
       <c r="FT59" s="54"/>
     </row>
-    <row r="60" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>59</v>
       </c>
@@ -5470,7 +5489,7 @@
         <v>14.998319755600814</v>
       </c>
     </row>
-    <row r="61" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>60</v>
       </c>
@@ -5488,7 +5507,7 @@
       </c>
       <c r="FT61" s="53"/>
     </row>
-    <row r="62" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>61</v>
       </c>
@@ -5511,7 +5530,7 @@
       </c>
       <c r="FT62" s="53"/>
     </row>
-    <row r="63" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>62</v>
       </c>
@@ -5531,7 +5550,7 @@
         <v>43.999616055846424</v>
       </c>
     </row>
-    <row r="64" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>63</v>
       </c>
@@ -5549,7 +5568,7 @@
       </c>
       <c r="FT64" s="53"/>
     </row>
-    <row r="65" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>64</v>
       </c>
@@ -5569,7 +5588,7 @@
         <v>4.0003912363067293</v>
       </c>
     </row>
-    <row r="66" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>65</v>
       </c>
@@ -5587,7 +5606,7 @@
       </c>
       <c r="FT66" s="53"/>
     </row>
-    <row r="67" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>66</v>
       </c>
@@ -5605,7 +5624,7 @@
       </c>
       <c r="FT67" s="53"/>
     </row>
-    <row r="68" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>67</v>
       </c>
@@ -5625,7 +5644,7 @@
         <v>3.9989973262032081</v>
       </c>
     </row>
-    <row r="69" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>68</v>
       </c>
@@ -5640,7 +5659,7 @@
       </c>
       <c r="FT69" s="53"/>
     </row>
-    <row r="70" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>69</v>
       </c>
@@ -5660,7 +5679,7 @@
         <v>29.998697867522175</v>
       </c>
     </row>
-    <row r="71" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>70</v>
       </c>
@@ -5679,7 +5698,7 @@
       </c>
       <c r="FT71" s="53"/>
     </row>
-    <row r="72" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>71</v>
       </c>
@@ -5697,7 +5716,7 @@
       </c>
       <c r="FT72" s="53"/>
     </row>
-    <row r="73" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
         <v>72</v>
       </c>
@@ -5717,7 +5736,7 @@
         <v>6.5296571480144401</v>
       </c>
     </row>
-    <row r="74" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
         <v>73</v>
       </c>
@@ -5737,7 +5756,7 @@
         <v>5.0005739365293724</v>
       </c>
     </row>
-    <row r="75" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
         <v>74</v>
       </c>
@@ -5753,11 +5772,12 @@
       <c r="BC75">
         <v>25</v>
       </c>
-      <c r="FT75" s="53">
-        <v>4.9996763754045306</v>
-      </c>
-    </row>
-    <row r="76" spans="1:176" x14ac:dyDescent="0.2">
+      <c r="FT75" s="60">
+        <f>AVERAGE(20,40)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="76" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
         <v>75</v>
       </c>
@@ -5776,7 +5796,7 @@
       </c>
       <c r="FT76" s="53"/>
     </row>
-    <row r="77" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
         <v>76</v>
       </c>
@@ -5793,7 +5813,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
         <v>77</v>
       </c>
@@ -5808,7 +5828,7 @@
       </c>
       <c r="FT78" s="53"/>
     </row>
-    <row r="79" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>78</v>
       </c>
@@ -5823,7 +5843,7 @@
       </c>
       <c r="FT79" s="53"/>
     </row>
-    <row r="80" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
         <v>79</v>
       </c>
@@ -5843,24 +5863,25 @@
         <v>40.999999999999993</v>
       </c>
     </row>
-    <row r="81" spans="1:199" s="60" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="59" t="s">
+    <row r="81" spans="1:199" x14ac:dyDescent="0.35">
+      <c r="A81" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B81" s="59" t="s">
+      <c r="B81" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="C81" s="59" t="s">
+      <c r="C81" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D81" s="59" t="s">
+      <c r="D81" s="2" t="s">
         <v>401</v>
       </c>
-      <c r="FT81" s="61">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82" spans="1:199" x14ac:dyDescent="0.2">
+      <c r="FT81" s="60">
+        <f>AVERAGE(30,50)</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="82" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
         <v>81</v>
       </c>
@@ -5875,7 +5896,7 @@
       </c>
       <c r="FT82" s="53"/>
     </row>
-    <row r="83" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>82</v>
       </c>
@@ -5890,7 +5911,7 @@
       </c>
       <c r="FT83" s="53"/>
     </row>
-    <row r="84" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
         <v>83</v>
       </c>
@@ -5910,7 +5931,7 @@
         <v>28.898261877172654</v>
       </c>
     </row>
-    <row r="85" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A85" s="2" t="s">
         <v>84</v>
       </c>
@@ -5930,7 +5951,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="86" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A86" s="2" t="s">
         <v>85</v>
       </c>
@@ -5950,7 +5971,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="87" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
         <v>86</v>
       </c>
@@ -5967,7 +5988,7 @@
         <v>12.5</v>
       </c>
     </row>
-    <row r="88" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
         <v>87</v>
       </c>
@@ -6035,7 +6056,7 @@
         <v>30.084</v>
       </c>
     </row>
-    <row r="89" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A89" s="2" t="s">
         <v>88</v>
       </c>
@@ -6055,7 +6076,7 @@
         <v>7.0002815957090174</v>
       </c>
     </row>
-    <row r="90" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A90" s="2" t="s">
         <v>89</v>
       </c>
@@ -6106,7 +6127,7 @@
         <v>9.1560000000000006</v>
       </c>
     </row>
-    <row r="91" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A91" s="2" t="s">
         <v>90</v>
       </c>
@@ -6126,7 +6147,7 @@
         <v>12.998784712675281</v>
       </c>
     </row>
-    <row r="92" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
         <v>91</v>
       </c>
@@ -6194,7 +6215,7 @@
         <v>11.336</v>
       </c>
     </row>
-    <row r="93" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
         <v>92</v>
       </c>
@@ -6214,7 +6235,7 @@
         <v>8.999644369178661</v>
       </c>
     </row>
-    <row r="94" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
         <v>93</v>
       </c>
@@ -6234,7 +6255,7 @@
         <v>13.999719192678953</v>
       </c>
     </row>
-    <row r="95" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A95" s="2" t="s">
         <v>94</v>
       </c>
@@ -6254,7 +6275,7 @@
         <v>23.99992076592935</v>
       </c>
     </row>
-    <row r="96" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A96" s="2" t="s">
         <v>95</v>
       </c>
@@ -6273,7 +6294,7 @@
       </c>
       <c r="FT96" s="53"/>
     </row>
-    <row r="97" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A97" s="2" t="s">
         <v>96</v>
       </c>
@@ -6320,7 +6341,7 @@
         <v>42.292000000000002</v>
       </c>
     </row>
-    <row r="98" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A98" s="2" t="s">
         <v>97</v>
       </c>
@@ -6339,7 +6360,7 @@
       </c>
       <c r="FT98" s="53"/>
     </row>
-    <row r="99" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A99" s="2" t="s">
         <v>98</v>
       </c>
@@ -6354,7 +6375,7 @@
       </c>
       <c r="FT99" s="53"/>
     </row>
-    <row r="100" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A100" s="2" t="s">
         <v>99</v>
       </c>
@@ -6374,7 +6395,7 @@
         <v>326.53131785066398</v>
       </c>
     </row>
-    <row r="101" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A101" s="2" t="s">
         <v>100</v>
       </c>
@@ -6392,7 +6413,7 @@
       </c>
       <c r="FT101" s="53"/>
     </row>
-    <row r="102" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A102" s="2" t="s">
         <v>101</v>
       </c>
@@ -6412,7 +6433,7 @@
         <v>40.99699192956713</v>
       </c>
     </row>
-    <row r="103" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
         <v>102</v>
       </c>
@@ -6427,7 +6448,7 @@
       </c>
       <c r="FT103" s="53"/>
     </row>
-    <row r="104" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
         <v>103</v>
       </c>
@@ -6442,7 +6463,7 @@
       </c>
       <c r="FT104" s="53"/>
     </row>
-    <row r="105" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A105" s="2" t="s">
         <v>104</v>
       </c>
@@ -6457,7 +6478,7 @@
       </c>
       <c r="FT105" s="53"/>
     </row>
-    <row r="106" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A106" s="2" t="s">
         <v>105</v>
       </c>
@@ -6477,7 +6498,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="107" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
         <v>106</v>
       </c>
@@ -6497,7 +6518,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="108" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
         <v>107</v>
       </c>
@@ -6517,37 +6538,37 @@
         <v>14</v>
       </c>
     </row>
-    <row r="109" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="2"/>
     </row>
-    <row r="110" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="2"/>
     </row>
-    <row r="111" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="2"/>
     </row>
-    <row r="112" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="2"/>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="2"/>
@@ -6564,20 +6585,20 @@
     <tabColor theme="6" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A2:GT115"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.33203125" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" customWidth="1"/>
-    <col min="5" max="202" width="5.6640625" customWidth="1"/>
+    <col min="2" max="2" width="32.90625" customWidth="1"/>
+    <col min="3" max="3" width="15.36328125" customWidth="1"/>
+    <col min="4" max="4" width="16.7265625" customWidth="1"/>
+    <col min="5" max="202" width="5.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:202" ht="19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:202" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A2" s="20" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="4" spans="1:202" ht="78.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:202" ht="78.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="22" t="s">
         <v>0</v>
       </c>
@@ -7178,7 +7199,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="5" spans="1:202" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:202" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="31" t="s">
         <v>1</v>
       </c>
@@ -7786,7 +7807,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="6" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -7809,7 +7830,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="7" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -7826,7 +7847,7 @@
       <c r="BC7" s="37"/>
       <c r="BD7" s="37"/>
     </row>
-    <row r="8" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -7846,7 +7867,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="9" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -7862,7 +7883,7 @@
       <c r="BC9" s="37"/>
       <c r="BD9" s="37"/>
     </row>
-    <row r="10" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -7882,7 +7903,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="11" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -7902,7 +7923,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="12" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -7918,7 +7939,7 @@
       <c r="BC12" s="40"/>
       <c r="BD12" s="40"/>
     </row>
-    <row r="13" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -7946,7 +7967,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="14" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -7962,7 +7983,7 @@
       <c r="BC14" s="38"/>
       <c r="BD14" s="39"/>
     </row>
-    <row r="15" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -7982,7 +8003,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="16" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:202" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -8002,7 +8023,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="17" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
@@ -8022,7 +8043,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="18" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
@@ -8042,7 +8063,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="19" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
@@ -8058,7 +8079,7 @@
       <c r="BC19" s="42"/>
       <c r="BD19" s="42"/>
     </row>
-    <row r="20" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
@@ -8078,7 +8099,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="21" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>19</v>
       </c>
@@ -8097,8 +8118,11 @@
       <c r="BD21" s="39" t="s">
         <v>665</v>
       </c>
-    </row>
-    <row r="22" spans="1:172" x14ac:dyDescent="0.2">
+      <c r="FT21" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="22" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -8117,8 +8141,11 @@
       <c r="BD22" s="39" t="s">
         <v>665</v>
       </c>
-    </row>
-    <row r="23" spans="1:172" x14ac:dyDescent="0.2">
+      <c r="FT22" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="23" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>21</v>
       </c>
@@ -8134,7 +8161,7 @@
       <c r="BC23" s="42"/>
       <c r="BD23" s="42"/>
     </row>
-    <row r="24" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>22</v>
       </c>
@@ -8153,8 +8180,11 @@
       <c r="BD24" s="39" t="s">
         <v>665</v>
       </c>
-    </row>
-    <row r="25" spans="1:172" x14ac:dyDescent="0.2">
+      <c r="FT24" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="25" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
@@ -8173,7 +8203,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="26" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
@@ -8192,8 +8222,11 @@
       <c r="BD26" s="39" t="s">
         <v>665</v>
       </c>
-    </row>
-    <row r="27" spans="1:172" x14ac:dyDescent="0.2">
+      <c r="FT26" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="27" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
@@ -8212,7 +8245,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="28" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
@@ -8231,8 +8264,11 @@
       <c r="BD28" s="39" t="s">
         <v>665</v>
       </c>
-    </row>
-    <row r="29" spans="1:172" x14ac:dyDescent="0.2">
+      <c r="FT28" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="29" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
@@ -8247,8 +8283,11 @@
       </c>
       <c r="BC29" s="37"/>
       <c r="BD29" s="37"/>
-    </row>
-    <row r="30" spans="1:172" x14ac:dyDescent="0.2">
+      <c r="FT29" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="30" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
@@ -8265,7 +8304,7 @@
       <c r="BC30" s="45"/>
       <c r="BD30" s="45"/>
     </row>
-    <row r="31" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>29</v>
       </c>
@@ -8281,7 +8320,7 @@
       <c r="BC31" s="45"/>
       <c r="BD31" s="45"/>
     </row>
-    <row r="32" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>30</v>
       </c>
@@ -8297,7 +8336,7 @@
       <c r="BC32" s="37"/>
       <c r="BD32" s="37"/>
     </row>
-    <row r="33" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>31</v>
       </c>
@@ -8316,7 +8355,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="34" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
@@ -8342,7 +8381,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="35" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>33</v>
       </c>
@@ -8367,7 +8406,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="36" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>34</v>
       </c>
@@ -8395,7 +8434,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="37" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>35</v>
       </c>
@@ -8415,7 +8454,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="38" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>36</v>
       </c>
@@ -8435,7 +8474,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="39" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>37</v>
       </c>
@@ -8455,7 +8494,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="40" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>38</v>
       </c>
@@ -8471,7 +8510,7 @@
       <c r="BC40" s="37"/>
       <c r="BD40" s="37"/>
     </row>
-    <row r="41" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>39</v>
       </c>
@@ -8491,7 +8530,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="42" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>40</v>
       </c>
@@ -8507,7 +8546,7 @@
       <c r="BC42" s="37"/>
       <c r="BD42" s="37"/>
     </row>
-    <row r="43" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>41</v>
       </c>
@@ -8523,7 +8562,7 @@
       <c r="BC43" s="40"/>
       <c r="BD43" s="40"/>
     </row>
-    <row r="44" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>42</v>
       </c>
@@ -8539,7 +8578,7 @@
       <c r="BC44" s="37"/>
       <c r="BD44" s="37"/>
     </row>
-    <row r="45" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>43</v>
       </c>
@@ -8555,7 +8594,7 @@
       <c r="BC45" s="37"/>
       <c r="BD45" s="37"/>
     </row>
-    <row r="46" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>44</v>
       </c>
@@ -8571,7 +8610,7 @@
       <c r="BC46" s="46"/>
       <c r="BD46" s="46"/>
     </row>
-    <row r="47" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>45</v>
       </c>
@@ -8587,7 +8626,7 @@
       <c r="BC47" s="45"/>
       <c r="BD47" s="45"/>
     </row>
-    <row r="48" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>46</v>
       </c>
@@ -8612,7 +8651,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="49" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>47</v>
       </c>
@@ -8628,7 +8667,7 @@
       <c r="BC49" s="45"/>
       <c r="BD49" s="45"/>
     </row>
-    <row r="50" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>48</v>
       </c>
@@ -8647,7 +8686,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="51" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>49</v>
       </c>
@@ -8666,8 +8705,11 @@
       <c r="BD51" s="39" t="s">
         <v>665</v>
       </c>
-    </row>
-    <row r="52" spans="1:176" x14ac:dyDescent="0.2">
+      <c r="FT51" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="52" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>50</v>
       </c>
@@ -8689,7 +8731,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="53" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>51</v>
       </c>
@@ -8705,7 +8747,7 @@
       <c r="BC53" s="45"/>
       <c r="BD53" s="45"/>
     </row>
-    <row r="54" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>52</v>
       </c>
@@ -8724,8 +8766,11 @@
       <c r="BD54" s="39" t="s">
         <v>665</v>
       </c>
-    </row>
-    <row r="55" spans="1:176" x14ac:dyDescent="0.2">
+      <c r="FT54" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="55" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>53</v>
       </c>
@@ -8741,7 +8786,7 @@
       <c r="BC55" s="45"/>
       <c r="BD55" s="45"/>
     </row>
-    <row r="56" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>54</v>
       </c>
@@ -8761,7 +8806,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="57" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>55</v>
       </c>
@@ -8781,7 +8826,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="58" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>56</v>
       </c>
@@ -8800,7 +8845,7 @@
       <c r="BC58" s="46"/>
       <c r="BD58" s="46"/>
     </row>
-    <row r="59" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>57</v>
       </c>
@@ -8819,7 +8864,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="60" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>59</v>
       </c>
@@ -8839,7 +8884,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="61" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>60</v>
       </c>
@@ -8858,7 +8903,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="62" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>61</v>
       </c>
@@ -8880,7 +8925,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="63" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>62</v>
       </c>
@@ -8900,7 +8945,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="64" spans="1:176" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>63</v>
       </c>
@@ -8919,7 +8964,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="65" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>64</v>
       </c>
@@ -8939,7 +8984,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="66" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>65</v>
       </c>
@@ -8959,7 +9004,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="67" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>66</v>
       </c>
@@ -8979,7 +9024,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="68" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>67</v>
       </c>
@@ -8999,7 +9044,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="69" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>68</v>
       </c>
@@ -9015,7 +9060,7 @@
       <c r="BC69" s="37"/>
       <c r="BD69" s="37"/>
     </row>
-    <row r="70" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>69</v>
       </c>
@@ -9035,7 +9080,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="71" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>70</v>
       </c>
@@ -9054,7 +9099,7 @@
       <c r="BC71" s="46"/>
       <c r="BD71" s="46"/>
     </row>
-    <row r="72" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>71</v>
       </c>
@@ -9073,7 +9118,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="73" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
         <v>72</v>
       </c>
@@ -9093,7 +9138,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="74" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
         <v>73</v>
       </c>
@@ -9113,7 +9158,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="75" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
         <v>74</v>
       </c>
@@ -9132,8 +9177,11 @@
       <c r="BD75" s="39" t="s">
         <v>665</v>
       </c>
-    </row>
-    <row r="76" spans="1:172" x14ac:dyDescent="0.2">
+      <c r="FT75" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="76" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
         <v>75</v>
       </c>
@@ -9152,7 +9200,7 @@
       <c r="BC76" s="46"/>
       <c r="BD76" s="46"/>
     </row>
-    <row r="77" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
         <v>76</v>
       </c>
@@ -9168,7 +9216,7 @@
       <c r="BC77" s="45"/>
       <c r="BD77" s="45"/>
     </row>
-    <row r="78" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
         <v>77</v>
       </c>
@@ -9184,7 +9232,7 @@
       <c r="BC78" s="45"/>
       <c r="BD78" s="45"/>
     </row>
-    <row r="79" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>78</v>
       </c>
@@ -9200,7 +9248,7 @@
       <c r="BC79" s="45"/>
       <c r="BD79" s="45"/>
     </row>
-    <row r="80" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
         <v>79</v>
       </c>
@@ -9220,7 +9268,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="81" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>80</v>
       </c>
@@ -9235,8 +9283,11 @@
       </c>
       <c r="BC81" s="37"/>
       <c r="BD81" s="37"/>
-    </row>
-    <row r="82" spans="1:199" x14ac:dyDescent="0.2">
+      <c r="FT81" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="82" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
         <v>81</v>
       </c>
@@ -9252,7 +9303,7 @@
       <c r="BC82" s="40"/>
       <c r="BD82" s="40"/>
     </row>
-    <row r="83" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>82</v>
       </c>
@@ -9268,7 +9319,7 @@
       <c r="BC83" s="46"/>
       <c r="BD83" s="46"/>
     </row>
-    <row r="84" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
         <v>83</v>
       </c>
@@ -9284,7 +9335,7 @@
       <c r="BC84" s="38"/>
       <c r="BD84" s="39"/>
     </row>
-    <row r="85" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A85" s="2" t="s">
         <v>84</v>
       </c>
@@ -9304,7 +9355,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="86" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A86" s="2" t="s">
         <v>85</v>
       </c>
@@ -9324,7 +9375,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="87" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
         <v>86</v>
       </c>
@@ -9340,7 +9391,7 @@
       <c r="BC87" s="37"/>
       <c r="BD87" s="37"/>
     </row>
-    <row r="88" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
         <v>87</v>
       </c>
@@ -9395,7 +9446,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="89" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A89" s="2" t="s">
         <v>88</v>
       </c>
@@ -9415,7 +9466,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="90" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A90" s="2" t="s">
         <v>89</v>
       </c>
@@ -9458,7 +9509,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="91" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A91" s="2" t="s">
         <v>90</v>
       </c>
@@ -9478,7 +9529,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="92" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
         <v>91</v>
       </c>
@@ -9534,7 +9585,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="93" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
         <v>92</v>
       </c>
@@ -9554,7 +9605,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="94" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
         <v>93</v>
       </c>
@@ -9574,7 +9625,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="95" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A95" s="2" t="s">
         <v>94</v>
       </c>
@@ -9594,7 +9645,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="96" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A96" s="2" t="s">
         <v>95</v>
       </c>
@@ -9613,7 +9664,7 @@
       <c r="BC96" s="45"/>
       <c r="BD96" s="45"/>
     </row>
-    <row r="97" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A97" s="2" t="s">
         <v>96</v>
       </c>
@@ -9654,7 +9705,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="98" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A98" s="2" t="s">
         <v>97</v>
       </c>
@@ -9673,7 +9724,7 @@
       <c r="BC98" s="48"/>
       <c r="BD98" s="48"/>
     </row>
-    <row r="99" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A99" s="2" t="s">
         <v>98</v>
       </c>
@@ -9689,7 +9740,7 @@
       <c r="BC99" s="45"/>
       <c r="BD99" s="45"/>
     </row>
-    <row r="100" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A100" s="2" t="s">
         <v>99</v>
       </c>
@@ -9709,7 +9760,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="101" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A101" s="2" t="s">
         <v>100</v>
       </c>
@@ -9729,7 +9780,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="102" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A102" s="2" t="s">
         <v>101</v>
       </c>
@@ -9749,7 +9800,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="103" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
         <v>102</v>
       </c>
@@ -9765,7 +9816,7 @@
       <c r="BC103" s="45"/>
       <c r="BD103" s="45"/>
     </row>
-    <row r="104" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
         <v>103</v>
       </c>
@@ -9781,7 +9832,7 @@
       <c r="BC104" s="49"/>
       <c r="BD104" s="49"/>
     </row>
-    <row r="105" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A105" s="2" t="s">
         <v>104</v>
       </c>
@@ -9797,7 +9848,7 @@
       <c r="BC105" s="50"/>
       <c r="BD105" s="50"/>
     </row>
-    <row r="106" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A106" s="2" t="s">
         <v>105</v>
       </c>
@@ -9813,7 +9864,7 @@
       <c r="BC106" s="38"/>
       <c r="BD106" s="39"/>
     </row>
-    <row r="107" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
         <v>106</v>
       </c>
@@ -9833,7 +9884,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="108" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
         <v>107</v>
       </c>
@@ -9853,37 +9904,37 @@
         <v>665</v>
       </c>
     </row>
-    <row r="109" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="2"/>
     </row>
-    <row r="110" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="2"/>
     </row>
-    <row r="111" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="2"/>
     </row>
-    <row r="112" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:190" x14ac:dyDescent="0.35">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="2"/>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="2"/>
@@ -9946,154 +9997,156 @@
     <tabColor theme="9" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A2:V42"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.33203125" style="4" customWidth="1"/>
-    <col min="2" max="4" width="8.6640625" style="4"/>
-    <col min="5" max="5" width="12.33203125" style="4" customWidth="1"/>
-    <col min="6" max="6" width="8.6640625" style="4"/>
-    <col min="7" max="7" width="8.6640625" style="4" customWidth="1"/>
-    <col min="8" max="16384" width="8.6640625" style="4"/>
+    <col min="1" max="1" width="10.36328125" style="4" customWidth="1"/>
+    <col min="2" max="4" width="8.6328125" style="4"/>
+    <col min="5" max="5" width="12.36328125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="8.6328125" style="4"/>
+    <col min="7" max="7" width="8.6328125" style="4" customWidth="1"/>
+    <col min="8" max="16384" width="8.6328125" style="4"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:22" ht="21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" ht="21" x14ac:dyDescent="0.5">
       <c r="A2" s="12" t="s">
         <v>679</v>
       </c>
     </row>
-    <row r="3" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="12"/>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>703</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>678</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>713</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>716</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>740</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A9" s="5"/>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>745</v>
+      </c>
       <c r="R9" s="11"/>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A10" s="10"/>
       <c r="V10" s="5"/>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A11" s="5"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A12" s="5"/>
       <c r="S12" s="9"/>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A13" s="7"/>
       <c r="S13" s="9"/>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A14" s="18"/>
       <c r="S14" s="9"/>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A15" s="5"/>
       <c r="S15" s="9"/>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A16" s="6"/>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A19" s="10"/>
       <c r="S19" s="9"/>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A20" s="8"/>
       <c r="R20" s="5"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A21" s="10"/>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A22" s="11"/>
       <c r="R22" s="5"/>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A23" s="11"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A24" s="5"/>
       <c r="V24" s="15"/>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A25" s="13"/>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A26" s="11"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A27" s="5"/>
       <c r="V27" s="5"/>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A28" s="5"/>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A29" s="10"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A30" s="10"/>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A31" s="10"/>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A32" s="10"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" s="10"/>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" s="10"/>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" s="16"/>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" s="5"/>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" s="14"/>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" s="5"/>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" s="10"/>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A42" s="17"/>
     </row>
   </sheetData>
@@ -10103,11 +10156,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10346,20 +10400,17 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{627ED23C-5EEB-4F10-AA20-79B788D8342E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A16A6EDB-4C6A-433C-9B54-BF88B9AEEE87}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10384,9 +10435,11 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A16A6EDB-4C6A-433C-9B54-BF88B9AEEE87}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{627ED23C-5EEB-4F10-AA20-79B788D8342E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>